<commit_message>
Пересобран fleet-trailers.xlsx: добавлен Makinsan L4 (makinsan-l4-pa066041)
</commit_message>
<xml_diff>
--- a/avito-feed-trailers/fleet-trailers.xlsx
+++ b/avito-feed-trailers/fleet-trailers.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BE19"/>
+  <dimension ref="A1:BE20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -1633,7 +1633,7 @@
       <c r="C7" s="1" t="inlineStr"/>
       <c r="D7" s="1" t="inlineStr">
         <is>
-          <t>steelbear-pf41n-v000319</t>
+          <t>makinsan-l4-pa066041</t>
         </is>
       </c>
       <c r="E7" s="1" t="inlineStr"/>
@@ -1650,12 +1650,11 @@
       </c>
       <c r="M7" s="1" t="inlineStr">
         <is>
-          <t>Полуприцеп-контейнеровоз Steelbear PF-41N (коммерческое название PF-41N FOX INTRA DISK), 4-х осный, универсал, под заказ.
-Перевозит 1×40-футовый контейнер (в т.ч. HQ), 2×20-футовых контейнера или 1×20-футовый по центру. Максимальная полная масса 47 000 кг, грузоподъёмность 41 100 кг, длина 12 600 мм.
-Осевой агрегат FOX B9-22S с дисковыми тормозами, допустимая нагрузка на ось 9 000 кг. Усиленная пневмоподвеска FOX INTRA с подъёмом/опусканием 1-й оси (ручное управление) и 2-й оси (автоматическое). Электронная тормозная система Haldex EBS 4S/2M с функцией противоопрокидывания (RSS), информационная система INFOCENTER.
-Опорное устройство GOS, 24 т, шкворень OREX 2 дюйма. Боковая алюминиевая защита, заднее защитное устройство. Два инструментальных ящика SKARB с замком. Шины TYREX 385/55R22,5 на дисках KRONPRINZ, 9 колёс в комплекте (включая запасное).
-При покупке в лизинг — скидка от Минпромторга 10%.
-Заводская гарантия — 12 месяцев. Поставка — 10 рабочих дней с момента предоплаты.</t>
+          <t>Полуприцеп-контейнеровоз Makinsan, универсальная платформа, 4 оси, 2023 год, в работе, полностью исправен.
+Оси SAF Intradisc 4×9 т с дисковыми тормозами — меньше износ и увереннее торможение в грузу. Пневматическая подвеска с подъёмом передней и задней оси — экономит резину и упрощает манёвры на порожняке. Тормозная система Wabco EBS 2S/2M со стояночным тормозом от энергоаккумуляторов, два противооткатных упора в комплекте.
+Шасси сварное, сталь ST52-3, изготовлено на роботизированном оборудовании — жёсткая рама под тяжёлые контейнерные перевозки. Опорный домкрат ОMS двухскоростной, 24 т. Электрика Aspock 24V по ECE R48, светодиодные фонари, два 7-контактных + один 15-контактный разъём.
+Грузоподъёмность 32 000 кг, разрешённая нагрузка на оси 36 000 кг, нагрузка на шкворень 11 000 кг. Общая длина 12 470 мм, снаряжённая масса 5 900 кг.
+Шины 385/55R22.5, комплект 8 колёс на стальных дисках.</t>
         </is>
       </c>
       <c r="N7" s="1" t="inlineStr">
@@ -1665,14 +1664,14 @@
       </c>
       <c r="O7" s="1" t="inlineStr">
         <is>
-          <t>3250000</t>
+          <t>2150000</t>
         </is>
       </c>
       <c r="P7" s="1" t="inlineStr"/>
       <c r="Q7" s="1" t="inlineStr"/>
       <c r="R7" s="1" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/steelbear-pf41n-v000319/01.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/steelbear-pf41n-v000319/02.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/steelbear-pf41n-v000319/03.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/steelbear-pf41n-v000319/04.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/steelbear-pf41n-v000319/05.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/steelbear-pf41n-v000319/06.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/steelbear-pf41n-v000319/07.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/steelbear-pf41n-v000319/08.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/steelbear-pf41n-v000319/09.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/steelbear-pf41n-v000319/10.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/steelbear-pf41n-v000319/11.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/steelbear-pf41n-v000319/12.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/steelbear-pf41n-v000319/13.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/steelbear-pf41n-v000319/14.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/steelbear-pf41n-v000319/15.jpg</t>
+          <t>https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/makinsan-l4-pa066041/01.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/makinsan-l4-pa066041/02.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/makinsan-l4-pa066041/03.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/makinsan-l4-pa066041/04.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/makinsan-l4-pa066041/05.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/makinsan-l4-pa066041/06.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/makinsan-l4-pa066041/07.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/makinsan-l4-pa066041/08.jpg</t>
         </is>
       </c>
       <c r="S7" s="1" t="inlineStr"/>
@@ -1702,19 +1701,15 @@
       <c r="AA7" s="1" t="inlineStr"/>
       <c r="AB7" s="1" t="inlineStr">
         <is>
-          <t>3250000</t>
+          <t>2150000</t>
         </is>
       </c>
       <c r="AC7" s="1" t="inlineStr">
         <is>
-          <t>Под заказ</t>
-        </is>
-      </c>
-      <c r="AD7" s="1" t="inlineStr">
-        <is>
-          <t>325000</t>
-        </is>
-      </c>
+          <t>В наличии</t>
+        </is>
+      </c>
+      <c r="AD7" s="1" t="inlineStr"/>
       <c r="AE7" s="1" t="inlineStr"/>
       <c r="AF7" s="1" t="inlineStr"/>
       <c r="AG7" s="1" t="inlineStr"/>
@@ -1725,7 +1720,7 @@
       <c r="AL7" s="1" t="inlineStr"/>
       <c r="AM7" s="1" t="inlineStr">
         <is>
-          <t>Новое</t>
+          <t>С пробегом</t>
         </is>
       </c>
       <c r="AN7" s="1" t="inlineStr"/>
@@ -1736,12 +1731,12 @@
       </c>
       <c r="AP7" s="1" t="inlineStr">
         <is>
-          <t>Steelbear</t>
+          <t>Makinsan</t>
         </is>
       </c>
       <c r="AQ7" s="1" t="inlineStr">
         <is>
-          <t>PF-41N</t>
+          <t>L4</t>
         </is>
       </c>
       <c r="AR7" s="1" t="inlineStr">
@@ -1756,10 +1751,14 @@
       </c>
       <c r="AT7" s="1" t="inlineStr"/>
       <c r="AU7" s="1" t="inlineStr"/>
-      <c r="AV7" s="1" t="inlineStr"/>
+      <c r="AV7" s="1" t="inlineStr">
+        <is>
+          <t>NP9L4CCP0PA066041</t>
+        </is>
+      </c>
       <c r="AW7" s="1" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>2023</t>
         </is>
       </c>
       <c r="AX7" s="1" t="inlineStr">
@@ -1779,12 +1778,12 @@
       </c>
       <c r="BA7" s="1" t="inlineStr">
         <is>
-          <t>41100</t>
+          <t>32000</t>
         </is>
       </c>
       <c r="BB7" s="1" t="inlineStr">
         <is>
-          <t>12600</t>
+          <t>12470</t>
         </is>
       </c>
       <c r="BC7" s="1" t="inlineStr"/>
@@ -1801,7 +1800,7 @@
       <c r="C8" s="1" t="inlineStr"/>
       <c r="D8" s="1" t="inlineStr">
         <is>
-          <t>steelbear-pl24l-avg36</t>
+          <t>steelbear-pf41n-v000319</t>
         </is>
       </c>
       <c r="E8" s="1" t="inlineStr"/>
@@ -1818,13 +1817,12 @@
       </c>
       <c r="M8" s="1" t="inlineStr">
         <is>
-          <t>Полуприцеп-сортиментовоз Steelbear PL-24L (коммерческое название PT-24L Fox), 3-х осный, под заказ.
-Осевой агрегат Fox, барабанные тормоза, допустимая нагрузка на ось 9 000 кг. Усиленная пневмоподвеска с подъёмом/опусканием. Электронная тормозная система TEBS 2S/2M с функцией противоопрокидывания (RSS), манометр давления в пневмоподвеске.
-6 пар коников с неоткрепляемыми стойками, грузоподъёмность 7 тонн каждая, положение регулируется вдоль рамы. Внутренняя высота коника 2 340 мм. 6 ремней для крепления сортимента. Неразборная передняя стенка перфорированного типа с крюками для каната и креплением для лома и лопаты.
-Опорное устройство GOS, 24 т, шкворень OREX 2 дюйма. Боковая алюминиевая противоподкатная защита. Металлический инструментальный ящик с замком. Шины TYREX 385/65R22,5.
-Максимальная полная масса 44 000 кг, грузоподъёмность 36 500 кг, длина 13 620 мм.
+          <t>Полуприцеп-контейнеровоз Steelbear PF-41N (коммерческое название PF-41N FOX INTRA DISK), 4-х осный, универсал, под заказ.
+Перевозит 1×40-футовый контейнер (в т.ч. HQ), 2×20-футовых контейнера или 1×20-футовый по центру. Максимальная полная масса 47 000 кг, грузоподъёмность 41 100 кг, длина 12 600 мм.
+Осевой агрегат FOX B9-22S с дисковыми тормозами, допустимая нагрузка на ось 9 000 кг. Усиленная пневмоподвеска FOX INTRA с подъёмом/опусканием 1-й оси (ручное управление) и 2-й оси (автоматическое). Электронная тормозная система Haldex EBS 4S/2M с функцией противоопрокидывания (RSS), информационная система INFOCENTER.
+Опорное устройство GOS, 24 т, шкворень OREX 2 дюйма. Боковая алюминиевая защита, заднее защитное устройство. Два инструментальных ящика SKARB с замком. Шины TYREX 385/55R22,5 на дисках KRONPRINZ, 9 колёс в комплекте (включая запасное).
 При покупке в лизинг — скидка от Минпромторга 10%.
-Заводская гарантия — 12 месяцев. Поставка — 15 рабочих дней с момента предоплаты.</t>
+Заводская гарантия — 12 месяцев. Поставка — 10 рабочих дней с момента предоплаты.</t>
         </is>
       </c>
       <c r="N8" s="1" t="inlineStr">
@@ -1834,14 +1832,14 @@
       </c>
       <c r="O8" s="1" t="inlineStr">
         <is>
-          <t>2960000</t>
+          <t>3250000</t>
         </is>
       </c>
       <c r="P8" s="1" t="inlineStr"/>
       <c r="Q8" s="1" t="inlineStr"/>
       <c r="R8" s="1" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/steelbear-pl24l-avg36/01.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/steelbear-pl24l-avg36/02.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/steelbear-pl24l-avg36/03.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/steelbear-pl24l-avg36/04.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/steelbear-pl24l-avg36/05.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/steelbear-pl24l-avg36/06.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/steelbear-pl24l-avg36/07.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/steelbear-pl24l-avg36/08.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/steelbear-pl24l-avg36/09.jpg</t>
+          <t>https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/steelbear-pf41n-v000319/01.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/steelbear-pf41n-v000319/02.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/steelbear-pf41n-v000319/03.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/steelbear-pf41n-v000319/04.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/steelbear-pf41n-v000319/05.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/steelbear-pf41n-v000319/06.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/steelbear-pf41n-v000319/07.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/steelbear-pf41n-v000319/08.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/steelbear-pf41n-v000319/09.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/steelbear-pf41n-v000319/10.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/steelbear-pf41n-v000319/11.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/steelbear-pf41n-v000319/12.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/steelbear-pf41n-v000319/13.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/steelbear-pf41n-v000319/14.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/steelbear-pf41n-v000319/15.jpg</t>
         </is>
       </c>
       <c r="S8" s="1" t="inlineStr"/>
@@ -1871,7 +1869,7 @@
       <c r="AA8" s="1" t="inlineStr"/>
       <c r="AB8" s="1" t="inlineStr">
         <is>
-          <t>2960000</t>
+          <t>3250000</t>
         </is>
       </c>
       <c r="AC8" s="1" t="inlineStr">
@@ -1881,7 +1879,7 @@
       </c>
       <c r="AD8" s="1" t="inlineStr">
         <is>
-          <t>296000</t>
+          <t>325000</t>
         </is>
       </c>
       <c r="AE8" s="1" t="inlineStr"/>
@@ -1910,7 +1908,7 @@
       </c>
       <c r="AQ8" s="1" t="inlineStr">
         <is>
-          <t>PL-24L</t>
+          <t>PF-41N</t>
         </is>
       </c>
       <c r="AR8" s="1" t="inlineStr">
@@ -1920,7 +1918,7 @@
       </c>
       <c r="AS8" s="1" t="inlineStr">
         <is>
-          <t>Лесовоз (сортиментовоз)</t>
+          <t>Контейнеровоз</t>
         </is>
       </c>
       <c r="AT8" s="1" t="inlineStr"/>
@@ -1933,7 +1931,7 @@
       </c>
       <c r="AX8" s="1" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="AY8" s="1" t="inlineStr">
@@ -1943,17 +1941,17 @@
       </c>
       <c r="AZ8" s="1" t="inlineStr">
         <is>
-          <t>Барабанные</t>
+          <t>Дисковые</t>
         </is>
       </c>
       <c r="BA8" s="1" t="inlineStr">
         <is>
-          <t>36500</t>
+          <t>41100</t>
         </is>
       </c>
       <c r="BB8" s="1" t="inlineStr">
         <is>
-          <t>13620</t>
+          <t>12600</t>
         </is>
       </c>
       <c r="BC8" s="1" t="inlineStr"/>
@@ -1970,7 +1968,7 @@
       <c r="C9" s="1" t="inlineStr"/>
       <c r="D9" s="1" t="inlineStr">
         <is>
-          <t>steelbear-pl24l-ea653666</t>
+          <t>steelbear-pl24l-avg36</t>
         </is>
       </c>
       <c r="E9" s="1" t="inlineStr"/>
@@ -1987,13 +1985,13 @@
       </c>
       <c r="M9" s="1" t="inlineStr">
         <is>
-          <t>Полуприцеп-сортиментовоз Steelbear PL-24L (коммерческое название PT-24L SAF Heavy Duty), 2024 год выпуска, б/у, в наличии.
-Усиленное шасси из двутавровых лонжеронов, 3 оси SAF Heavy Duty, барабанные тормоза, пневмоподвеска с функцией подъём/опускание, допустимая нагрузка на ось 9 000 кг. Шины 385/65R22,5, односкат. Электронная тормозная система WABCO TEBS-E с функцией противоопрокидывания (RSS).
-6 пар открепляемых коников грузоподъёмностью 8 тонн каждая (сталь STRENX 700MC), положение регулируется вдоль рамы. Внутренняя высота коника 2330 мм. Настил из ламинированной берёзовой фанеры. Опорное устройство BPW, 24 т.
-Максимальная полная масса 44 000 кг, грузоподъёмность 37 100 кг, длина 13 620 мм.
-Техническое состояние — на ходу, полностью исправен, не требует вложений и ремонта.
-Документы в порядке.
-Смотровая площадка и показ — по договорённости. Торг при осмотре.</t>
+          <t>Полуприцеп-сортиментовоз Steelbear PL-24L (коммерческое название PT-24L Fox), 3-х осный, под заказ.
+Осевой агрегат Fox, барабанные тормоза, допустимая нагрузка на ось 9 000 кг. Усиленная пневмоподвеска с подъёмом/опусканием. Электронная тормозная система TEBS 2S/2M с функцией противоопрокидывания (RSS), манометр давления в пневмоподвеске.
+6 пар коников с неоткрепляемыми стойками, грузоподъёмность 7 тонн каждая, положение регулируется вдоль рамы. Внутренняя высота коника 2 340 мм. 6 ремней для крепления сортимента. Неразборная передняя стенка перфорированного типа с крюками для каната и креплением для лома и лопаты.
+Опорное устройство GOS, 24 т, шкворень OREX 2 дюйма. Боковая алюминиевая противоподкатная защита. Металлический инструментальный ящик с замком. Шины TYREX 385/65R22,5.
+Максимальная полная масса 44 000 кг, грузоподъёмность 36 500 кг, длина 13 620 мм.
+При покупке в лизинг — скидка от Минпромторга 10%.
+Заводская гарантия — 12 месяцев. Поставка — 15 рабочих дней с момента предоплаты.</t>
         </is>
       </c>
       <c r="N9" s="1" t="inlineStr">
@@ -2003,14 +2001,14 @@
       </c>
       <c r="O9" s="1" t="inlineStr">
         <is>
-          <t>2970000</t>
+          <t>2960000</t>
         </is>
       </c>
       <c r="P9" s="1" t="inlineStr"/>
       <c r="Q9" s="1" t="inlineStr"/>
       <c r="R9" s="1" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/steelbear-pl24l-ea653666/01.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/steelbear-pl24l-ea653666/02.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/steelbear-pl24l-ea653666/03.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/steelbear-pl24l-ea653666/04.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/steelbear-pl24l-ea653666/05.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/steelbear-pl24l-ea653666/06.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/steelbear-pl24l-ea653666/07.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/steelbear-pl24l-ea653666/08.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/steelbear-pl24l-ea653666/09.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/steelbear-pl24l-ea653666/10.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/steelbear-pl24l-ea653666/11.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/steelbear-pl24l-ea653666/12.jpg</t>
+          <t>https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/steelbear-pl24l-avg36/01.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/steelbear-pl24l-avg36/02.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/steelbear-pl24l-avg36/03.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/steelbear-pl24l-avg36/04.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/steelbear-pl24l-avg36/05.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/steelbear-pl24l-avg36/06.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/steelbear-pl24l-avg36/07.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/steelbear-pl24l-avg36/08.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/steelbear-pl24l-avg36/09.jpg</t>
         </is>
       </c>
       <c r="S9" s="1" t="inlineStr"/>
@@ -2040,7 +2038,7 @@
       <c r="AA9" s="1" t="inlineStr"/>
       <c r="AB9" s="1" t="inlineStr">
         <is>
-          <t>2970000</t>
+          <t>2960000</t>
         </is>
       </c>
       <c r="AC9" s="1" t="inlineStr">
@@ -2048,7 +2046,11 @@
           <t>Под заказ</t>
         </is>
       </c>
-      <c r="AD9" s="1" t="inlineStr"/>
+      <c r="AD9" s="1" t="inlineStr">
+        <is>
+          <t>296000</t>
+        </is>
+      </c>
       <c r="AE9" s="1" t="inlineStr"/>
       <c r="AF9" s="1" t="inlineStr"/>
       <c r="AG9" s="1" t="inlineStr"/>
@@ -2059,7 +2061,7 @@
       <c r="AL9" s="1" t="inlineStr"/>
       <c r="AM9" s="1" t="inlineStr">
         <is>
-          <t>С пробегом</t>
+          <t>Новое</t>
         </is>
       </c>
       <c r="AN9" s="1" t="inlineStr"/>
@@ -2090,14 +2092,10 @@
       </c>
       <c r="AT9" s="1" t="inlineStr"/>
       <c r="AU9" s="1" t="inlineStr"/>
-      <c r="AV9" s="1" t="inlineStr">
-        <is>
-          <t>XWZ9412LLR1202021</t>
-        </is>
-      </c>
+      <c r="AV9" s="1" t="inlineStr"/>
       <c r="AW9" s="1" t="inlineStr">
         <is>
-          <t>2024</t>
+          <t>2026</t>
         </is>
       </c>
       <c r="AX9" s="1" t="inlineStr">
@@ -2117,7 +2115,7 @@
       </c>
       <c r="BA9" s="1" t="inlineStr">
         <is>
-          <t>37100</t>
+          <t>36500</t>
         </is>
       </c>
       <c r="BB9" s="1" t="inlineStr">
@@ -2139,7 +2137,7 @@
       <c r="C10" s="1" t="inlineStr"/>
       <c r="D10" s="1" t="inlineStr">
         <is>
-          <t>tonar-b313-9888</t>
+          <t>steelbear-pl24l-ea653666</t>
         </is>
       </c>
       <c r="E10" s="1" t="inlineStr"/>
@@ -2156,12 +2154,13 @@
       </c>
       <c r="M10" s="1" t="inlineStr">
         <is>
-          <t>Полуприцеп бортовой Тонар B3-13 (9888), 13,6 м, трёхосный, первая ось подъёмная — меньше износ резины на порожняке. ССУ 1200 мм, со стаканами под коники (коники в комплект не входят). Новое, под заказ у завода-изготовителя.
-Цена по действующему прайсу завода (с 27.07.2026): 3 150 000 ₽.
-Скидка от производителя на линейку бортовых прицепов (10%): −315 000 ₽.
-При покупке в лизинг — дополнительная субсидия от Минпромторга (10%, не более 500 000 ₽): −315 000 ₽.
-Итоговая цена при лизинге: 2 520 000 ₽.
-Заводская гарантия — 12 месяцев. Поставка после согласования комплектации.</t>
+          <t>Полуприцеп-сортиментовоз Steelbear PL-24L (коммерческое название PT-24L SAF Heavy Duty), 2024 год выпуска, б/у, в наличии.
+Усиленное шасси из двутавровых лонжеронов, 3 оси SAF Heavy Duty, барабанные тормоза, пневмоподвеска с функцией подъём/опускание, допустимая нагрузка на ось 9 000 кг. Шины 385/65R22,5, односкат. Электронная тормозная система WABCO TEBS-E с функцией противоопрокидывания (RSS).
+6 пар открепляемых коников грузоподъёмностью 8 тонн каждая (сталь STRENX 700MC), положение регулируется вдоль рамы. Внутренняя высота коника 2330 мм. Настил из ламинированной берёзовой фанеры. Опорное устройство BPW, 24 т.
+Максимальная полная масса 44 000 кг, грузоподъёмность 37 100 кг, длина 13 620 мм.
+Техническое состояние — на ходу, полностью исправен, не требует вложений и ремонта.
+Документы в порядке.
+Смотровая площадка и показ — по договорённости. Торг при осмотре.</t>
         </is>
       </c>
       <c r="N10" s="1" t="inlineStr">
@@ -2171,14 +2170,14 @@
       </c>
       <c r="O10" s="1" t="inlineStr">
         <is>
-          <t>3150000</t>
+          <t>2970000</t>
         </is>
       </c>
       <c r="P10" s="1" t="inlineStr"/>
       <c r="Q10" s="1" t="inlineStr"/>
       <c r="R10" s="1" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-b313-9888/01.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-b313-9888/02.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-b313-9888/03.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-b313-9888/04.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-b313-9888/05.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-b313-9888/06.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-b313-9888/07.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-b313-9888/08.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-b313-9888/09.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-b313-9888/10.jpg</t>
+          <t>https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/steelbear-pl24l-ea653666/01.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/steelbear-pl24l-ea653666/02.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/steelbear-pl24l-ea653666/03.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/steelbear-pl24l-ea653666/04.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/steelbear-pl24l-ea653666/05.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/steelbear-pl24l-ea653666/06.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/steelbear-pl24l-ea653666/07.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/steelbear-pl24l-ea653666/08.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/steelbear-pl24l-ea653666/09.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/steelbear-pl24l-ea653666/10.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/steelbear-pl24l-ea653666/11.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/steelbear-pl24l-ea653666/12.jpg</t>
         </is>
       </c>
       <c r="S10" s="1" t="inlineStr"/>
@@ -2208,7 +2207,7 @@
       <c r="AA10" s="1" t="inlineStr"/>
       <c r="AB10" s="1" t="inlineStr">
         <is>
-          <t>3150000</t>
+          <t>2970000</t>
         </is>
       </c>
       <c r="AC10" s="1" t="inlineStr">
@@ -2216,17 +2215,9 @@
           <t>Под заказ</t>
         </is>
       </c>
-      <c r="AD10" s="1" t="inlineStr">
-        <is>
-          <t>315000</t>
-        </is>
-      </c>
+      <c r="AD10" s="1" t="inlineStr"/>
       <c r="AE10" s="1" t="inlineStr"/>
-      <c r="AF10" s="1" t="inlineStr">
-        <is>
-          <t>315000</t>
-        </is>
-      </c>
+      <c r="AF10" s="1" t="inlineStr"/>
       <c r="AG10" s="1" t="inlineStr"/>
       <c r="AH10" s="1" t="inlineStr"/>
       <c r="AI10" s="1" t="inlineStr"/>
@@ -2235,7 +2226,7 @@
       <c r="AL10" s="1" t="inlineStr"/>
       <c r="AM10" s="1" t="inlineStr">
         <is>
-          <t>Новое</t>
+          <t>С пробегом</t>
         </is>
       </c>
       <c r="AN10" s="1" t="inlineStr"/>
@@ -2246,12 +2237,12 @@
       </c>
       <c r="AP10" s="1" t="inlineStr">
         <is>
-          <t>Тонар</t>
+          <t>Steelbear</t>
         </is>
       </c>
       <c r="AQ10" s="1" t="inlineStr">
         <is>
-          <t>B3-13 (9888)</t>
+          <t>PL-24L</t>
         </is>
       </c>
       <c r="AR10" s="1" t="inlineStr">
@@ -2261,15 +2252,19 @@
       </c>
       <c r="AS10" s="1" t="inlineStr">
         <is>
-          <t>Бортовой</t>
+          <t>Лесовоз (сортиментовоз)</t>
         </is>
       </c>
       <c r="AT10" s="1" t="inlineStr"/>
       <c r="AU10" s="1" t="inlineStr"/>
-      <c r="AV10" s="1" t="inlineStr"/>
+      <c r="AV10" s="1" t="inlineStr">
+        <is>
+          <t>XWZ9412LLR1202021</t>
+        </is>
+      </c>
       <c r="AW10" s="1" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>2024</t>
         </is>
       </c>
       <c r="AX10" s="1" t="inlineStr">
@@ -2289,12 +2284,12 @@
       </c>
       <c r="BA10" s="1" t="inlineStr">
         <is>
-          <t>31600</t>
+          <t>37100</t>
         </is>
       </c>
       <c r="BB10" s="1" t="inlineStr">
         <is>
-          <t>13600</t>
+          <t>13620</t>
         </is>
       </c>
       <c r="BC10" s="1" t="inlineStr"/>
@@ -2311,7 +2306,7 @@
       <c r="C11" s="1" t="inlineStr"/>
       <c r="D11" s="1" t="inlineStr">
         <is>
-          <t>tonar-k4u-99891-order</t>
+          <t>tonar-b313-9888</t>
         </is>
       </c>
       <c r="E11" s="1" t="inlineStr"/>
@@ -2328,13 +2323,12 @@
       </c>
       <c r="M11" s="1" t="inlineStr">
         <is>
-          <t>Полуприцеп контейнеровоз Тонар K4-U (99891), 4 оси, вынесенная вперёд передняя ось на 2560 мм — меньше нагрузка на дорогу. ССУ=1100 мм, шины 385/55-R22.5. Берёт контейнеры 1×20', 2×20', 1×30', 1×40' High Cube. Новое, под заказ у завода-изготовителя.
-Цена по действующему прайсу завода (с 27.07.2026): 3 200 000 ₽.
-Скидка от производителя на линейку контейнеровозов (5%): −160 000 ₽.
-При покупке в лизинг — дополнительная субсидия от Минпромторга (10%, не более 500 000 ₽): −320 000 ₽.
-Итоговая цена при лизинге: 2 720 000 ₽.
-Заводская гарантия — 12 месяцев. Поставка после согласования комплектации.
-(У нас также есть эта же модель б/у, в наличии, дешевле — уточняйте по телефону, если новый под заказ не подходит по срокам.)</t>
+          <t>Полуприцеп бортовой Тонар B3-13 (9888), 13,6 м, трёхосный, первая ось подъёмная — меньше износ резины на порожняке. ССУ 1200 мм, со стаканами под коники (коники в комплект не входят). Новое, под заказ у завода-изготовителя.
+Цена по действующему прайсу завода (с 27.07.2026): 3 150 000 ₽.
+Скидка от производителя на линейку бортовых прицепов (10%): −315 000 ₽.
+При покупке в лизинг — дополнительная субсидия от Минпромторга (10%, не более 500 000 ₽): −315 000 ₽.
+Итоговая цена при лизинге: 2 520 000 ₽.
+Заводская гарантия — 12 месяцев. Поставка после согласования комплектации.</t>
         </is>
       </c>
       <c r="N11" s="1" t="inlineStr">
@@ -2344,14 +2338,14 @@
       </c>
       <c r="O11" s="1" t="inlineStr">
         <is>
-          <t>3200000</t>
+          <t>3150000</t>
         </is>
       </c>
       <c r="P11" s="1" t="inlineStr"/>
       <c r="Q11" s="1" t="inlineStr"/>
       <c r="R11" s="1" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-k4u-99891-order/01.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-k4u-99891-order/02.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-k4u-99891-order/03.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-k4u-99891-order/04.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-k4u-99891-order/05.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-k4u-99891-order/06.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-k4u-99891-order/07.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-k4u-99891-order/08.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-k4u-99891-order/09.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-k4u-99891-order/10.jpg</t>
+          <t>https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-b313-9888/01.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-b313-9888/02.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-b313-9888/03.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-b313-9888/04.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-b313-9888/05.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-b313-9888/06.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-b313-9888/07.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-b313-9888/08.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-b313-9888/09.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-b313-9888/10.jpg</t>
         </is>
       </c>
       <c r="S11" s="1" t="inlineStr"/>
@@ -2381,7 +2375,7 @@
       <c r="AA11" s="1" t="inlineStr"/>
       <c r="AB11" s="1" t="inlineStr">
         <is>
-          <t>3200000</t>
+          <t>3150000</t>
         </is>
       </c>
       <c r="AC11" s="1" t="inlineStr">
@@ -2391,13 +2385,13 @@
       </c>
       <c r="AD11" s="1" t="inlineStr">
         <is>
-          <t>320000</t>
+          <t>315000</t>
         </is>
       </c>
       <c r="AE11" s="1" t="inlineStr"/>
       <c r="AF11" s="1" t="inlineStr">
         <is>
-          <t>160000</t>
+          <t>315000</t>
         </is>
       </c>
       <c r="AG11" s="1" t="inlineStr"/>
@@ -2424,7 +2418,7 @@
       </c>
       <c r="AQ11" s="1" t="inlineStr">
         <is>
-          <t>K4-U (99891)</t>
+          <t>B3-13 (9888)</t>
         </is>
       </c>
       <c r="AR11" s="1" t="inlineStr">
@@ -2434,7 +2428,7 @@
       </c>
       <c r="AS11" s="1" t="inlineStr">
         <is>
-          <t>Контейнеровоз</t>
+          <t>Бортовой</t>
         </is>
       </c>
       <c r="AT11" s="1" t="inlineStr"/>
@@ -2447,7 +2441,7 @@
       </c>
       <c r="AX11" s="1" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="AY11" s="1" t="inlineStr">
@@ -2462,12 +2456,12 @@
       </c>
       <c r="BA11" s="1" t="inlineStr">
         <is>
-          <t>37800</t>
+          <t>31600</t>
         </is>
       </c>
       <c r="BB11" s="1" t="inlineStr">
         <is>
-          <t>12192</t>
+          <t>13600</t>
         </is>
       </c>
       <c r="BC11" s="1" t="inlineStr"/>
@@ -2484,7 +2478,7 @@
       <c r="C12" s="1" t="inlineStr"/>
       <c r="D12" s="1" t="inlineStr">
         <is>
-          <t>tonar-k4u-p0002033</t>
+          <t>tonar-k4u-99891-order</t>
         </is>
       </c>
       <c r="E12" s="1" t="inlineStr"/>
@@ -2501,10 +2495,13 @@
       </c>
       <c r="M12" s="1" t="inlineStr">
         <is>
-          <t>Полуприцеп-контейнеровоз Тонар К4-U (99891), 2023 год, в работе, полностью исправен.
-4 оси: тройная задняя тележка плюс вынесенная вперёд ось — меньше нагрузка на дорогу и мягче по осевым ограничениям в городе. Тормоза дисковые, пневмопривод. Подвеска зависимая, на продольных рычагах, с пневмоэлементами и телескопическими амортизаторами. Шины 385/55R22.5, односкатные.
-Берёт контейнеры 20', 2×20', 30', 30' HC, 40', 40' HC. Разрешённая максимальная масса 44 000 кг, грузоподъёмность 37 800 кг, нагрузка на ССУ 11 000 кг. Высота ССУ 1 100 мм.
-Возможна аренда с правом выкупа — уточняйте условия по телефону.</t>
+          <t>Полуприцеп контейнеровоз Тонар K4-U (99891), 4 оси, вынесенная вперёд передняя ось на 2560 мм — меньше нагрузка на дорогу. ССУ=1100 мм, шины 385/55-R22.5. Берёт контейнеры 1×20', 2×20', 1×30', 1×40' High Cube. Новое, под заказ у завода-изготовителя.
+Цена по действующему прайсу завода (с 27.07.2026): 3 200 000 ₽.
+Скидка от производителя на линейку контейнеровозов (5%): −160 000 ₽.
+При покупке в лизинг — дополнительная субсидия от Минпромторга (10%, не более 500 000 ₽): −320 000 ₽.
+Итоговая цена при лизинге: 2 720 000 ₽.
+Заводская гарантия — 12 месяцев. Поставка после согласования комплектации.
+(У нас также есть эта же модель б/у, в наличии, дешевле — уточняйте по телефону, если новый под заказ не подходит по срокам.)</t>
         </is>
       </c>
       <c r="N12" s="1" t="inlineStr">
@@ -2514,14 +2511,14 @@
       </c>
       <c r="O12" s="1" t="inlineStr">
         <is>
-          <t>1690000</t>
+          <t>3200000</t>
         </is>
       </c>
       <c r="P12" s="1" t="inlineStr"/>
       <c r="Q12" s="1" t="inlineStr"/>
       <c r="R12" s="1" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-k4u-p0002033/01.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-k4u-p0002033/02.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-k4u-p0002033/03.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-k4u-p0002033/04.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-k4u-p0002033/05.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-k4u-p0002033/06.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-k4u-p0002033/07.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-k4u-p0002033/08.jpg</t>
+          <t>https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-k4u-99891-order/01.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-k4u-99891-order/02.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-k4u-99891-order/03.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-k4u-99891-order/04.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-k4u-99891-order/05.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-k4u-99891-order/06.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-k4u-99891-order/07.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-k4u-99891-order/08.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-k4u-99891-order/09.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-k4u-99891-order/10.jpg</t>
         </is>
       </c>
       <c r="S12" s="1" t="inlineStr"/>
@@ -2551,7 +2548,7 @@
       <c r="AA12" s="1" t="inlineStr"/>
       <c r="AB12" s="1" t="inlineStr">
         <is>
-          <t>1690000</t>
+          <t>3200000</t>
         </is>
       </c>
       <c r="AC12" s="1" t="inlineStr">
@@ -2559,9 +2556,17 @@
           <t>Под заказ</t>
         </is>
       </c>
-      <c r="AD12" s="1" t="inlineStr"/>
+      <c r="AD12" s="1" t="inlineStr">
+        <is>
+          <t>320000</t>
+        </is>
+      </c>
       <c r="AE12" s="1" t="inlineStr"/>
-      <c r="AF12" s="1" t="inlineStr"/>
+      <c r="AF12" s="1" t="inlineStr">
+        <is>
+          <t>160000</t>
+        </is>
+      </c>
       <c r="AG12" s="1" t="inlineStr"/>
       <c r="AH12" s="1" t="inlineStr"/>
       <c r="AI12" s="1" t="inlineStr"/>
@@ -2570,7 +2575,7 @@
       <c r="AL12" s="1" t="inlineStr"/>
       <c r="AM12" s="1" t="inlineStr">
         <is>
-          <t>С пробегом</t>
+          <t>Новое</t>
         </is>
       </c>
       <c r="AN12" s="1" t="inlineStr"/>
@@ -2601,14 +2606,10 @@
       </c>
       <c r="AT12" s="1" t="inlineStr"/>
       <c r="AU12" s="1" t="inlineStr"/>
-      <c r="AV12" s="1" t="inlineStr">
-        <is>
-          <t>X0T998910P0002033</t>
-        </is>
-      </c>
+      <c r="AV12" s="1" t="inlineStr"/>
       <c r="AW12" s="1" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2026</t>
         </is>
       </c>
       <c r="AX12" s="1" t="inlineStr">
@@ -2618,12 +2619,12 @@
       </c>
       <c r="AY12" s="1" t="inlineStr">
         <is>
-          <t>Рессорная</t>
+          <t>Пневматическая</t>
         </is>
       </c>
       <c r="AZ12" s="1" t="inlineStr">
         <is>
-          <t>Дисковые</t>
+          <t>Барабанные</t>
         </is>
       </c>
       <c r="BA12" s="1" t="inlineStr">
@@ -2633,7 +2634,7 @@
       </c>
       <c r="BB12" s="1" t="inlineStr">
         <is>
-          <t>12725</t>
+          <t>12192</t>
         </is>
       </c>
       <c r="BC12" s="1" t="inlineStr"/>
@@ -2650,7 +2651,7 @@
       <c r="C13" s="1" t="inlineStr"/>
       <c r="D13" s="1" t="inlineStr">
         <is>
-          <t>tonar-l3-9445</t>
+          <t>tonar-k4u-p0002033</t>
         </is>
       </c>
       <c r="E13" s="1" t="inlineStr"/>
@@ -2667,12 +2668,10 @@
       </c>
       <c r="M13" s="1" t="inlineStr">
         <is>
-          <t>Полуприцеп-сортиментовоз Тонар L3 (9445), 3 оси, ССУ 1150/1250/1350 мм с подъёмной осью — меньше износ на порожняке. Коники разборные, 6 штук, межосевое расстояние 1310 мм, рычажная подвеска, барабанные тормоза. Новое, под заказ у завода-изготовителя.
-Цена по действующему прайсу завода (с 27.07.2026): 3 200 000 ₽.
-Скидка от производителя на линейку лесовозов (5%): −160 000 ₽.
-При покупке в лизинг — дополнительная субсидия от Минпромторга (10%, не более 500 000 ₽): −320 000 ₽.
-Итоговая цена при лизинге: 2 720 000 ₽.
-Заводская гарантия — 12 месяцев. Поставка после согласования комплектации.</t>
+          <t>Полуприцеп-контейнеровоз Тонар К4-U (99891), 2023 год, в работе, полностью исправен.
+4 оси: тройная задняя тележка плюс вынесенная вперёд ось — меньше нагрузка на дорогу и мягче по осевым ограничениям в городе. Тормоза дисковые, пневмопривод. Подвеска зависимая, на продольных рычагах, с пневмоэлементами и телескопическими амортизаторами. Шины 385/55R22.5, односкатные.
+Берёт контейнеры 20', 2×20', 30', 30' HC, 40', 40' HC. Разрешённая максимальная масса 44 000 кг, грузоподъёмность 37 800 кг, нагрузка на ССУ 11 000 кг. Высота ССУ 1 100 мм.
+Возможна аренда с правом выкупа — уточняйте условия по телефону.</t>
         </is>
       </c>
       <c r="N13" s="1" t="inlineStr">
@@ -2682,14 +2681,14 @@
       </c>
       <c r="O13" s="1" t="inlineStr">
         <is>
-          <t>3200000</t>
+          <t>1690000</t>
         </is>
       </c>
       <c r="P13" s="1" t="inlineStr"/>
       <c r="Q13" s="1" t="inlineStr"/>
       <c r="R13" s="1" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-l3-9445/01.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-l3-9445/02.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-l3-9445/03.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-l3-9445/04.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-l3-9445/05.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-l3-9445/06.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-l3-9445/07.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-l3-9445/08.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-l3-9445/09.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-l3-9445/10.jpg</t>
+          <t>https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-k4u-p0002033/01.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-k4u-p0002033/02.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-k4u-p0002033/03.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-k4u-p0002033/04.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-k4u-p0002033/05.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-k4u-p0002033/06.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-k4u-p0002033/07.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-k4u-p0002033/08.jpg</t>
         </is>
       </c>
       <c r="S13" s="1" t="inlineStr"/>
@@ -2719,7 +2718,7 @@
       <c r="AA13" s="1" t="inlineStr"/>
       <c r="AB13" s="1" t="inlineStr">
         <is>
-          <t>3200000</t>
+          <t>1690000</t>
         </is>
       </c>
       <c r="AC13" s="1" t="inlineStr">
@@ -2727,17 +2726,9 @@
           <t>Под заказ</t>
         </is>
       </c>
-      <c r="AD13" s="1" t="inlineStr">
-        <is>
-          <t>320000</t>
-        </is>
-      </c>
+      <c r="AD13" s="1" t="inlineStr"/>
       <c r="AE13" s="1" t="inlineStr"/>
-      <c r="AF13" s="1" t="inlineStr">
-        <is>
-          <t>160000</t>
-        </is>
-      </c>
+      <c r="AF13" s="1" t="inlineStr"/>
       <c r="AG13" s="1" t="inlineStr"/>
       <c r="AH13" s="1" t="inlineStr"/>
       <c r="AI13" s="1" t="inlineStr"/>
@@ -2746,7 +2737,7 @@
       <c r="AL13" s="1" t="inlineStr"/>
       <c r="AM13" s="1" t="inlineStr">
         <is>
-          <t>Новое</t>
+          <t>С пробегом</t>
         </is>
       </c>
       <c r="AN13" s="1" t="inlineStr"/>
@@ -2762,7 +2753,7 @@
       </c>
       <c r="AQ13" s="1" t="inlineStr">
         <is>
-          <t>L3 (9445)</t>
+          <t>K4-U (99891)</t>
         </is>
       </c>
       <c r="AR13" s="1" t="inlineStr">
@@ -2772,47 +2763,47 @@
       </c>
       <c r="AS13" s="1" t="inlineStr">
         <is>
-          <t>Лесовоз (сортиментовоз)</t>
+          <t>Контейнеровоз</t>
         </is>
       </c>
       <c r="AT13" s="1" t="inlineStr"/>
       <c r="AU13" s="1" t="inlineStr"/>
-      <c r="AV13" s="1" t="inlineStr"/>
+      <c r="AV13" s="1" t="inlineStr">
+        <is>
+          <t>X0T998910P0002033</t>
+        </is>
+      </c>
       <c r="AW13" s="1" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>2023</t>
         </is>
       </c>
       <c r="AX13" s="1" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="AY13" s="1" t="inlineStr">
         <is>
-          <t>Пневматическая</t>
+          <t>Рессорная</t>
         </is>
       </c>
       <c r="AZ13" s="1" t="inlineStr">
         <is>
-          <t>Барабанные</t>
+          <t>Дисковые</t>
         </is>
       </c>
       <c r="BA13" s="1" t="inlineStr">
         <is>
-          <t>36700</t>
+          <t>37800</t>
         </is>
       </c>
       <c r="BB13" s="1" t="inlineStr">
         <is>
-          <t>12800</t>
-        </is>
-      </c>
-      <c r="BC13" s="1" t="inlineStr">
-        <is>
-          <t>63</t>
-        </is>
-      </c>
+          <t>12725</t>
+        </is>
+      </c>
+      <c r="BC13" s="1" t="inlineStr"/>
       <c r="BD13" s="1" t="inlineStr"/>
       <c r="BE13" s="1" t="inlineStr"/>
     </row>
@@ -2826,7 +2817,7 @@
       <c r="C14" s="1" t="inlineStr"/>
       <c r="D14" s="1" t="inlineStr">
         <is>
-          <t>tonar-reef-r313</t>
+          <t>tonar-l3-9445</t>
         </is>
       </c>
       <c r="E14" s="1" t="inlineStr"/>
@@ -2843,11 +2834,11 @@
       </c>
       <c r="M14" s="1" t="inlineStr">
         <is>
-          <t>Полуприцеп рефрижератор Тонар R3-13, 13,6 м, трёхосный, первая ось подъёмная, объём кузова 85 м³, дисковые оси, ССУ-1150 мм, вместимость 33 европаллеты. Новое, под заказ у завода-изготовителя.
-В отличие от обычного изотермического кузова (без активного охлаждения), этот прицеп доукомплектован новой холодильно-отопительной установкой (ХОУ) — держит заданную температуру в пути, не только теплоизолирует. Именно установка ХОУ и делает цену заметно выше базового изотермического кузова той же длины (у нас в парке такой есть от 4 850 000 ₽ по прайсу завода без холодильной установки).
-Цена: 7 365 000 ₽ (на эту линейку скидка от производителя не действует).
-При покупке в лизинг — субсидия от Минпромторга (10%, не более 500 000 ₽): −500 000 ₽.
-Итоговая цена при лизинге: 6 865 000 ₽.
+          <t>Полуприцеп-сортиментовоз Тонар L3 (9445), 3 оси, ССУ 1150/1250/1350 мм с подъёмной осью — меньше износ на порожняке. Коники разборные, 6 штук, межосевое расстояние 1310 мм, рычажная подвеска, барабанные тормоза. Новое, под заказ у завода-изготовителя.
+Цена по действующему прайсу завода (с 27.07.2026): 3 200 000 ₽.
+Скидка от производителя на линейку лесовозов (5%): −160 000 ₽.
+При покупке в лизинг — дополнительная субсидия от Минпромторга (10%, не более 500 000 ₽): −320 000 ₽.
+Итоговая цена при лизинге: 2 720 000 ₽.
 Заводская гарантия — 12 месяцев. Поставка после согласования комплектации.</t>
         </is>
       </c>
@@ -2858,14 +2849,14 @@
       </c>
       <c r="O14" s="1" t="inlineStr">
         <is>
-          <t>7365000</t>
+          <t>3200000</t>
         </is>
       </c>
       <c r="P14" s="1" t="inlineStr"/>
       <c r="Q14" s="1" t="inlineStr"/>
       <c r="R14" s="1" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-reef-r313/r2-01.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-reef-r313/06.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-reef-r313/r2-07.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-reef-r313/05.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-reef-r313/02.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-reef-r313/03.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-reef-r313/08.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-reef-r313/04.jpg</t>
+          <t>https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-l3-9445/01.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-l3-9445/02.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-l3-9445/03.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-l3-9445/04.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-l3-9445/05.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-l3-9445/06.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-l3-9445/07.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-l3-9445/08.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-l3-9445/09.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-l3-9445/10.jpg</t>
         </is>
       </c>
       <c r="S14" s="1" t="inlineStr"/>
@@ -2895,7 +2886,7 @@
       <c r="AA14" s="1" t="inlineStr"/>
       <c r="AB14" s="1" t="inlineStr">
         <is>
-          <t>7365000</t>
+          <t>3200000</t>
         </is>
       </c>
       <c r="AC14" s="1" t="inlineStr">
@@ -2905,11 +2896,15 @@
       </c>
       <c r="AD14" s="1" t="inlineStr">
         <is>
-          <t>500000</t>
+          <t>320000</t>
         </is>
       </c>
       <c r="AE14" s="1" t="inlineStr"/>
-      <c r="AF14" s="1" t="inlineStr"/>
+      <c r="AF14" s="1" t="inlineStr">
+        <is>
+          <t>160000</t>
+        </is>
+      </c>
       <c r="AG14" s="1" t="inlineStr"/>
       <c r="AH14" s="1" t="inlineStr"/>
       <c r="AI14" s="1" t="inlineStr"/>
@@ -2934,7 +2929,7 @@
       </c>
       <c r="AQ14" s="1" t="inlineStr">
         <is>
-          <t>R3-13</t>
+          <t>L3 (9445)</t>
         </is>
       </c>
       <c r="AR14" s="1" t="inlineStr">
@@ -2944,7 +2939,7 @@
       </c>
       <c r="AS14" s="1" t="inlineStr">
         <is>
-          <t>Рефрижератор</t>
+          <t>Лесовоз (сортиментовоз)</t>
         </is>
       </c>
       <c r="AT14" s="1" t="inlineStr"/>
@@ -2967,22 +2962,22 @@
       </c>
       <c r="AZ14" s="1" t="inlineStr">
         <is>
-          <t>Дисковые</t>
+          <t>Барабанные</t>
         </is>
       </c>
       <c r="BA14" s="1" t="inlineStr">
         <is>
-          <t>31200</t>
+          <t>36700</t>
         </is>
       </c>
       <c r="BB14" s="1" t="inlineStr">
         <is>
-          <t>13600</t>
+          <t>12800</t>
         </is>
       </c>
       <c r="BC14" s="1" t="inlineStr">
         <is>
-          <t>85</t>
+          <t>63</t>
         </is>
       </c>
       <c r="BD14" s="1" t="inlineStr"/>
@@ -2998,7 +2993,7 @@
       <c r="C15" s="1" t="inlineStr"/>
       <c r="D15" s="1" t="inlineStr">
         <is>
-          <t>tonar-samosval-9595</t>
+          <t>tonar-reef-r313</t>
         </is>
       </c>
       <c r="E15" s="1" t="inlineStr"/>
@@ -3015,10 +3010,11 @@
       </c>
       <c r="M15" s="1" t="inlineStr">
         <is>
-          <t>Полуприцеп самосвальный Тонар SH4-34 (9595) с задней разгрузкой, облегчённый, объём кузова 33,6 м³, четырёхосный, пневматическая рычажная подвеска, барабанные тормоза. Кузов полукруглой формы — сыпучий груз сходит легче, без залипания, в том числе влажный. Подходит под сыпучие строительные материалы. Тент с ручной намоткой в базе. Новое, под заказ у завода-изготовителя.
-Цена: 4 200 000 ₽ (на линейку самосвальных полуприцепов скидка от производителя не действует).
-При покупке в лизинг — субсидия от Минпромторга (10%, не более 500 000 ₽): −420 000 ₽.
-Итоговая цена при лизинге: 3 780 000 ₽.
+          <t>Полуприцеп рефрижератор Тонар R3-13, 13,6 м, трёхосный, первая ось подъёмная, объём кузова 85 м³, дисковые оси, ССУ-1150 мм, вместимость 33 европаллеты. Новое, под заказ у завода-изготовителя.
+В отличие от обычного изотермического кузова (без активного охлаждения), этот прицеп доукомплектован новой холодильно-отопительной установкой (ХОУ) — держит заданную температуру в пути, не только теплоизолирует. Именно установка ХОУ и делает цену заметно выше базового изотермического кузова той же длины (у нас в парке такой есть от 4 850 000 ₽ по прайсу завода без холодильной установки).
+Цена: 7 365 000 ₽ (на эту линейку скидка от производителя не действует).
+При покупке в лизинг — субсидия от Минпромторга (10%, не более 500 000 ₽): −500 000 ₽.
+Итоговая цена при лизинге: 6 865 000 ₽.
 Заводская гарантия — 12 месяцев. Поставка после согласования комплектации.</t>
         </is>
       </c>
@@ -3029,14 +3025,14 @@
       </c>
       <c r="O15" s="1" t="inlineStr">
         <is>
-          <t>4200000</t>
+          <t>7365000</t>
         </is>
       </c>
       <c r="P15" s="1" t="inlineStr"/>
       <c r="Q15" s="1" t="inlineStr"/>
       <c r="R15" s="1" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-samosval-9595/01.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-samosval-9595/02.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-samosval-9595/03.jpg</t>
+          <t>https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-reef-r313/r2-01.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-reef-r313/06.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-reef-r313/r2-07.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-reef-r313/05.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-reef-r313/02.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-reef-r313/03.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-reef-r313/08.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-reef-r313/04.jpg</t>
         </is>
       </c>
       <c r="S15" s="1" t="inlineStr"/>
@@ -3066,7 +3062,7 @@
       <c r="AA15" s="1" t="inlineStr"/>
       <c r="AB15" s="1" t="inlineStr">
         <is>
-          <t>4200000</t>
+          <t>7365000</t>
         </is>
       </c>
       <c r="AC15" s="1" t="inlineStr">
@@ -3076,7 +3072,7 @@
       </c>
       <c r="AD15" s="1" t="inlineStr">
         <is>
-          <t>420000</t>
+          <t>500000</t>
         </is>
       </c>
       <c r="AE15" s="1" t="inlineStr"/>
@@ -3105,7 +3101,7 @@
       </c>
       <c r="AQ15" s="1" t="inlineStr">
         <is>
-          <t>9595</t>
+          <t>R3-13</t>
         </is>
       </c>
       <c r="AR15" s="1" t="inlineStr">
@@ -3115,7 +3111,7 @@
       </c>
       <c r="AS15" s="1" t="inlineStr">
         <is>
-          <t>Самосвальный</t>
+          <t>Рефрижератор</t>
         </is>
       </c>
       <c r="AT15" s="1" t="inlineStr"/>
@@ -3128,7 +3124,7 @@
       </c>
       <c r="AX15" s="1" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="AY15" s="1" t="inlineStr">
@@ -3138,18 +3134,22 @@
       </c>
       <c r="AZ15" s="1" t="inlineStr">
         <is>
-          <t>Барабанные</t>
+          <t>Дисковые</t>
         </is>
       </c>
       <c r="BA15" s="1" t="inlineStr">
         <is>
-          <t>30000</t>
-        </is>
-      </c>
-      <c r="BB15" s="1" t="inlineStr"/>
+          <t>31200</t>
+        </is>
+      </c>
+      <c r="BB15" s="1" t="inlineStr">
+        <is>
+          <t>13600</t>
+        </is>
+      </c>
       <c r="BC15" s="1" t="inlineStr">
         <is>
-          <t>33.6</t>
+          <t>85</t>
         </is>
       </c>
       <c r="BD15" s="1" t="inlineStr"/>
@@ -3165,7 +3165,7 @@
       <c r="C16" s="1" t="inlineStr"/>
       <c r="D16" s="1" t="inlineStr">
         <is>
-          <t>tonar-sdp489-95895</t>
+          <t>tonar-samosval-9595</t>
         </is>
       </c>
       <c r="E16" s="1" t="inlineStr"/>
@@ -3182,11 +3182,10 @@
       </c>
       <c r="M16" s="1" t="inlineStr">
         <is>
-          <t>Полуприцеп со сдвижными полами Тонар SDP4-89 (95895), 4 оси (первая вынесенная), габаритная длина 14,6 м, погрузочная длина 14,1 м, алюминиевый кузов, объём 89 м³, ССУ=1150 мм. Новое, под заказ у завода-изготовителя.
-Сдвижной пол (Cargo Floor) выгружает груз горизонтально, без опрокидывания кузова — можно разгружаться на неровных площадках и под низкими навесами, где самосвал не встанет. Универсален под насыпные грузы: щепа, зерно, песок и т.п.
-Цена: 7 650 000 ₽ (на эту линейку скидка от производителя не действует).
-При покупке в лизинг — субсидия от Минпромторга (10%, не более 500 000 ₽): −500 000 ₽.
-Итоговая цена при лизинге: 7 150 000 ₽.
+          <t>Полуприцеп самосвальный Тонар SH4-34 (9595) с задней разгрузкой, облегчённый, объём кузова 33,6 м³, четырёхосный, пневматическая рычажная подвеска, барабанные тормоза. Кузов полукруглой формы — сыпучий груз сходит легче, без залипания, в том числе влажный. Подходит под сыпучие строительные материалы. Тент с ручной намоткой в базе. Новое, под заказ у завода-изготовителя.
+Цена: 4 200 000 ₽ (на линейку самосвальных полуприцепов скидка от производителя не действует).
+При покупке в лизинг — субсидия от Минпромторга (10%, не более 500 000 ₽): −420 000 ₽.
+Итоговая цена при лизинге: 3 780 000 ₽.
 Заводская гарантия — 12 месяцев. Поставка после согласования комплектации.</t>
         </is>
       </c>
@@ -3197,14 +3196,14 @@
       </c>
       <c r="O16" s="1" t="inlineStr">
         <is>
-          <t>7650000</t>
+          <t>4200000</t>
         </is>
       </c>
       <c r="P16" s="1" t="inlineStr"/>
       <c r="Q16" s="1" t="inlineStr"/>
       <c r="R16" s="1" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-sdp489-95895/01.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-sdp489-95895/02.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-sdp489-95895/03.jpg</t>
+          <t>https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-samosval-9595/01.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-samosval-9595/02.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-samosval-9595/03.jpg</t>
         </is>
       </c>
       <c r="S16" s="1" t="inlineStr"/>
@@ -3234,7 +3233,7 @@
       <c r="AA16" s="1" t="inlineStr"/>
       <c r="AB16" s="1" t="inlineStr">
         <is>
-          <t>7650000</t>
+          <t>4200000</t>
         </is>
       </c>
       <c r="AC16" s="1" t="inlineStr">
@@ -3244,7 +3243,7 @@
       </c>
       <c r="AD16" s="1" t="inlineStr">
         <is>
-          <t>500000</t>
+          <t>420000</t>
         </is>
       </c>
       <c r="AE16" s="1" t="inlineStr"/>
@@ -3273,7 +3272,7 @@
       </c>
       <c r="AQ16" s="1" t="inlineStr">
         <is>
-          <t>SDP4-89 (95895)</t>
+          <t>9595</t>
         </is>
       </c>
       <c r="AR16" s="1" t="inlineStr">
@@ -3283,7 +3282,7 @@
       </c>
       <c r="AS16" s="1" t="inlineStr">
         <is>
-          <t>Щеповоз</t>
+          <t>Самосвальный</t>
         </is>
       </c>
       <c r="AT16" s="1" t="inlineStr"/>
@@ -3306,22 +3305,18 @@
       </c>
       <c r="AZ16" s="1" t="inlineStr">
         <is>
-          <t>Дисковые</t>
+          <t>Барабанные</t>
         </is>
       </c>
       <c r="BA16" s="1" t="inlineStr">
         <is>
-          <t>27800</t>
-        </is>
-      </c>
-      <c r="BB16" s="1" t="inlineStr">
-        <is>
-          <t>14600</t>
-        </is>
-      </c>
+          <t>30000</t>
+        </is>
+      </c>
+      <c r="BB16" s="1" t="inlineStr"/>
       <c r="BC16" s="1" t="inlineStr">
         <is>
-          <t>89.6</t>
+          <t>33.6</t>
         </is>
       </c>
       <c r="BD16" s="1" t="inlineStr"/>
@@ -3337,7 +3332,7 @@
       <c r="C17" s="1" t="inlineStr"/>
       <c r="D17" s="1" t="inlineStr">
         <is>
-          <t>tonar-t313-9888</t>
+          <t>tonar-sdp489-95895</t>
         </is>
       </c>
       <c r="E17" s="1" t="inlineStr"/>
@@ -3354,11 +3349,11 @@
       </c>
       <c r="M17" s="1" t="inlineStr">
         <is>
-          <t>Полуприцеп шторно-бортовой Тонар T3-13 (9888), 13,6 м, трёхосный, первая ось подъёмная, объём 91,4 м³. Дисковые оси, ССУ-1150 мм, со стаканами под коники (коники в комплект не входят). Новое, под заказ у завода-изготовителя.
-Цена по действующему прайсу завода (с 27.07.2026): 3 800 000 ₽.
-Скидка от производителя на линейку шторных прицепов (10%): −380 000 ₽.
-При покупке в лизинг — дополнительная субсидия от Минпромторга (10%, не более 500 000 ₽): −380 000 ₽.
-Итоговая цена при лизинге: 3 040 000 ₽.
+          <t>Полуприцеп со сдвижными полами Тонар SDP4-89 (95895), 4 оси (первая вынесенная), габаритная длина 14,6 м, погрузочная длина 14,1 м, алюминиевый кузов, объём 89 м³, ССУ=1150 мм. Новое, под заказ у завода-изготовителя.
+Сдвижной пол (Cargo Floor) выгружает груз горизонтально, без опрокидывания кузова — можно разгружаться на неровных площадках и под низкими навесами, где самосвал не встанет. Универсален под насыпные грузы: щепа, зерно, песок и т.п.
+Цена: 7 650 000 ₽ (на эту линейку скидка от производителя не действует).
+При покупке в лизинг — субсидия от Минпромторга (10%, не более 500 000 ₽): −500 000 ₽.
+Итоговая цена при лизинге: 7 150 000 ₽.
 Заводская гарантия — 12 месяцев. Поставка после согласования комплектации.</t>
         </is>
       </c>
@@ -3369,14 +3364,14 @@
       </c>
       <c r="O17" s="1" t="inlineStr">
         <is>
-          <t>3800000</t>
+          <t>7650000</t>
         </is>
       </c>
       <c r="P17" s="1" t="inlineStr"/>
       <c r="Q17" s="1" t="inlineStr"/>
       <c r="R17" s="1" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-t313-9888/01.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-t313-9888/02.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-t313-9888/03.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-t313-9888/04.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-t313-9888/05.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-t313-9888/06.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-t313-9888/07.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-t313-9888/08.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-t313-9888/09.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-t313-9888/10.jpg</t>
+          <t>https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-sdp489-95895/01.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-sdp489-95895/02.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-sdp489-95895/03.jpg</t>
         </is>
       </c>
       <c r="S17" s="1" t="inlineStr"/>
@@ -3406,7 +3401,7 @@
       <c r="AA17" s="1" t="inlineStr"/>
       <c r="AB17" s="1" t="inlineStr">
         <is>
-          <t>3800000</t>
+          <t>7650000</t>
         </is>
       </c>
       <c r="AC17" s="1" t="inlineStr">
@@ -3416,15 +3411,11 @@
       </c>
       <c r="AD17" s="1" t="inlineStr">
         <is>
-          <t>380000</t>
+          <t>500000</t>
         </is>
       </c>
       <c r="AE17" s="1" t="inlineStr"/>
-      <c r="AF17" s="1" t="inlineStr">
-        <is>
-          <t>380000</t>
-        </is>
-      </c>
+      <c r="AF17" s="1" t="inlineStr"/>
       <c r="AG17" s="1" t="inlineStr"/>
       <c r="AH17" s="1" t="inlineStr"/>
       <c r="AI17" s="1" t="inlineStr"/>
@@ -3449,7 +3440,7 @@
       </c>
       <c r="AQ17" s="1" t="inlineStr">
         <is>
-          <t>T3-13 (9888)</t>
+          <t>SDP4-89 (95895)</t>
         </is>
       </c>
       <c r="AR17" s="1" t="inlineStr">
@@ -3459,7 +3450,7 @@
       </c>
       <c r="AS17" s="1" t="inlineStr">
         <is>
-          <t>Шторно-бортовой</t>
+          <t>Щеповоз</t>
         </is>
       </c>
       <c r="AT17" s="1" t="inlineStr"/>
@@ -3472,7 +3463,7 @@
       </c>
       <c r="AX17" s="1" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="AY17" s="1" t="inlineStr">
@@ -3487,17 +3478,17 @@
       </c>
       <c r="BA17" s="1" t="inlineStr">
         <is>
-          <t>31000</t>
+          <t>27800</t>
         </is>
       </c>
       <c r="BB17" s="1" t="inlineStr">
         <is>
-          <t>13600</t>
+          <t>14600</t>
         </is>
       </c>
       <c r="BC17" s="1" t="inlineStr">
         <is>
-          <t>91.4</t>
+          <t>89.6</t>
         </is>
       </c>
       <c r="BD17" s="1" t="inlineStr"/>
@@ -3513,7 +3504,7 @@
       <c r="C18" s="1" t="inlineStr"/>
       <c r="D18" s="1" t="inlineStr">
         <is>
-          <t>tonar-zernovoz-95941</t>
+          <t>tonar-t313-9888</t>
         </is>
       </c>
       <c r="E18" s="1" t="inlineStr"/>
@@ -3530,10 +3521,11 @@
       </c>
       <c r="M18" s="1" t="inlineStr">
         <is>
-          <t>Полуприцеп-зерновоз Тонар 95941 с задней разгрузкой, алюминиевый кузов прямоугольной формы, объём 50 м³, до 31 тонны груза. Тент с механическим приводом в базовой комплектации. Задний борт комбинированный (откидной и распашной), с разгрузочными люками. Подвеска рычажного типа с пневмоэлементами, 3 оси (первая подъёмная), тормозная система TEBS. Универсален — насыпные зерновые/комбикорм и паллетированный груз. Новое, под заказ у завода-изготовителя.
-Цена: 5 400 000 ₽ (на линейку зерновозов скидка от производителя не действует).
-При покупке в лизинг — субсидия от Минпромторга (10%, не более 500 000 ₽): −500 000 ₽.
-Итоговая цена при лизинге: 4 900 000 ₽.
+          <t>Полуприцеп шторно-бортовой Тонар T3-13 (9888), 13,6 м, трёхосный, первая ось подъёмная, объём 91,4 м³. Дисковые оси, ССУ-1150 мм, со стаканами под коники (коники в комплект не входят). Новое, под заказ у завода-изготовителя.
+Цена по действующему прайсу завода (с 27.07.2026): 3 800 000 ₽.
+Скидка от производителя на линейку шторных прицепов (10%): −380 000 ₽.
+При покупке в лизинг — дополнительная субсидия от Минпромторга (10%, не более 500 000 ₽): −380 000 ₽.
+Итоговая цена при лизинге: 3 040 000 ₽.
 Заводская гарантия — 12 месяцев. Поставка после согласования комплектации.</t>
         </is>
       </c>
@@ -3544,14 +3536,14 @@
       </c>
       <c r="O18" s="1" t="inlineStr">
         <is>
-          <t>5400000</t>
+          <t>3800000</t>
         </is>
       </c>
       <c r="P18" s="1" t="inlineStr"/>
       <c r="Q18" s="1" t="inlineStr"/>
       <c r="R18" s="1" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-zernovoz-95941/01.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-zernovoz-95941/02.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-zernovoz-95941/03.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-zernovoz-95941/04.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-zernovoz-95941/05.jpg</t>
+          <t>https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-t313-9888/01.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-t313-9888/02.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-t313-9888/03.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-t313-9888/04.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-t313-9888/05.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-t313-9888/06.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-t313-9888/07.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-t313-9888/08.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-t313-9888/09.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-t313-9888/10.jpg</t>
         </is>
       </c>
       <c r="S18" s="1" t="inlineStr"/>
@@ -3581,7 +3573,7 @@
       <c r="AA18" s="1" t="inlineStr"/>
       <c r="AB18" s="1" t="inlineStr">
         <is>
-          <t>5400000</t>
+          <t>3800000</t>
         </is>
       </c>
       <c r="AC18" s="1" t="inlineStr">
@@ -3591,11 +3583,15 @@
       </c>
       <c r="AD18" s="1" t="inlineStr">
         <is>
-          <t>500000</t>
+          <t>380000</t>
         </is>
       </c>
       <c r="AE18" s="1" t="inlineStr"/>
-      <c r="AF18" s="1" t="inlineStr"/>
+      <c r="AF18" s="1" t="inlineStr">
+        <is>
+          <t>380000</t>
+        </is>
+      </c>
       <c r="AG18" s="1" t="inlineStr"/>
       <c r="AH18" s="1" t="inlineStr"/>
       <c r="AI18" s="1" t="inlineStr"/>
@@ -3620,7 +3616,7 @@
       </c>
       <c r="AQ18" s="1" t="inlineStr">
         <is>
-          <t>95941</t>
+          <t>T3-13 (9888)</t>
         </is>
       </c>
       <c r="AR18" s="1" t="inlineStr">
@@ -3630,7 +3626,7 @@
       </c>
       <c r="AS18" s="1" t="inlineStr">
         <is>
-          <t>Зерновоз</t>
+          <t>Шторно-бортовой</t>
         </is>
       </c>
       <c r="AT18" s="1" t="inlineStr"/>
@@ -3653,7 +3649,7 @@
       </c>
       <c r="AZ18" s="1" t="inlineStr">
         <is>
-          <t>Барабанные</t>
+          <t>Дисковые</t>
         </is>
       </c>
       <c r="BA18" s="1" t="inlineStr">
@@ -3661,10 +3657,14 @@
           <t>31000</t>
         </is>
       </c>
-      <c r="BB18" s="1" t="inlineStr"/>
+      <c r="BB18" s="1" t="inlineStr">
+        <is>
+          <t>13600</t>
+        </is>
+      </c>
       <c r="BC18" s="1" t="inlineStr">
         <is>
-          <t>50</t>
+          <t>91.4</t>
         </is>
       </c>
       <c r="BD18" s="1" t="inlineStr"/>
@@ -3680,7 +3680,7 @@
       <c r="C19" s="1" t="inlineStr"/>
       <c r="D19" s="1" t="inlineStr">
         <is>
-          <t>v-trailer-329d-r0000119</t>
+          <t>tonar-zernovoz-95941</t>
         </is>
       </c>
       <c r="E19" s="1" t="inlineStr"/>
@@ -3697,10 +3697,11 @@
       </c>
       <c r="M19" s="1" t="inlineStr">
         <is>
-          <t>Шторный полуприцеп V-Trailer 329D, 2023 год, в работе, полностью исправен.
-Оси SAF, подъёмная передняя — меньше износ резины и расход на порожняке. Опорное устройство JOST на 24 тонны, шкворень 2 дюйма по ISO 1726. Пол — влагостойкая фанера 30 мм, держит погрузчик до 7,5 тонн. Крыша сдвижная (Sesam/Edscha) — грузить сверху краном или погрузчиком без снятия тента. Двери алюминиевые BPW Smartmaster II, передний и задний портал — стальные, собственной конструкции. Рама облегчённая, с дополнительными усилениями против скручивания. По бортам — корзины под коники, по 7 штук на сторону.
-13,6 × 2,5 × 4 м, 91 м³. Тент плотный: борта 900 г/м², крыша 680 г/м². Полная штора, без бортов — удобно под европаллеты и груз с выступом по высоте.
-Возможна аренда с правом выкупа — уточняйте условия по телефону.</t>
+          <t>Полуприцеп-зерновоз Тонар 95941 с задней разгрузкой, алюминиевый кузов прямоугольной формы, объём 50 м³, до 31 тонны груза. Тент с механическим приводом в базовой комплектации. Задний борт комбинированный (откидной и распашной), с разгрузочными люками. Подвеска рычажного типа с пневмоэлементами, 3 оси (первая подъёмная), тормозная система TEBS. Универсален — насыпные зерновые/комбикорм и паллетированный груз. Новое, под заказ у завода-изготовителя.
+Цена: 5 400 000 ₽ (на линейку зерновозов скидка от производителя не действует).
+При покупке в лизинг — субсидия от Минпромторга (10%, не более 500 000 ₽): −500 000 ₽.
+Итоговая цена при лизинге: 4 900 000 ₽.
+Заводская гарантия — 12 месяцев. Поставка после согласования комплектации.</t>
         </is>
       </c>
       <c r="N19" s="1" t="inlineStr">
@@ -3710,14 +3711,14 @@
       </c>
       <c r="O19" s="1" t="inlineStr">
         <is>
-          <t>2990000</t>
+          <t>5400000</t>
         </is>
       </c>
       <c r="P19" s="1" t="inlineStr"/>
       <c r="Q19" s="1" t="inlineStr"/>
       <c r="R19" s="1" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/v-trailer-329d-r0000119/r2-01.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/v-trailer-329d-r0000119/r2-02.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/v-trailer-329d-r0000119/r2-03.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/v-trailer-329d-r0000119/r2-04.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/v-trailer-329d-r0000119/r2-05.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/v-trailer-329d-r0000119/r2-06.jpg</t>
+          <t>https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-zernovoz-95941/01.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-zernovoz-95941/02.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-zernovoz-95941/03.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-zernovoz-95941/04.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/tonar-zernovoz-95941/05.jpg</t>
         </is>
       </c>
       <c r="S19" s="1" t="inlineStr"/>
@@ -3747,7 +3748,7 @@
       <c r="AA19" s="1" t="inlineStr"/>
       <c r="AB19" s="1" t="inlineStr">
         <is>
-          <t>2990000</t>
+          <t>5400000</t>
         </is>
       </c>
       <c r="AC19" s="1" t="inlineStr">
@@ -3755,7 +3756,11 @@
           <t>Под заказ</t>
         </is>
       </c>
-      <c r="AD19" s="1" t="inlineStr"/>
+      <c r="AD19" s="1" t="inlineStr">
+        <is>
+          <t>500000</t>
+        </is>
+      </c>
       <c r="AE19" s="1" t="inlineStr"/>
       <c r="AF19" s="1" t="inlineStr"/>
       <c r="AG19" s="1" t="inlineStr"/>
@@ -3766,7 +3771,7 @@
       <c r="AL19" s="1" t="inlineStr"/>
       <c r="AM19" s="1" t="inlineStr">
         <is>
-          <t>С пробегом</t>
+          <t>Новое</t>
         </is>
       </c>
       <c r="AN19" s="1" t="inlineStr"/>
@@ -3777,12 +3782,12 @@
       </c>
       <c r="AP19" s="1" t="inlineStr">
         <is>
-          <t>V-Trailer</t>
+          <t>Тонар</t>
         </is>
       </c>
       <c r="AQ19" s="1" t="inlineStr">
         <is>
-          <t>329</t>
+          <t>95941</t>
         </is>
       </c>
       <c r="AR19" s="1" t="inlineStr">
@@ -3792,19 +3797,15 @@
       </c>
       <c r="AS19" s="1" t="inlineStr">
         <is>
-          <t>Шторный</t>
+          <t>Зерновоз</t>
         </is>
       </c>
       <c r="AT19" s="1" t="inlineStr"/>
       <c r="AU19" s="1" t="inlineStr"/>
-      <c r="AV19" s="1" t="inlineStr">
-        <is>
-          <t>XZFVKRP3DR0000119</t>
-        </is>
-      </c>
+      <c r="AV19" s="1" t="inlineStr"/>
       <c r="AW19" s="1" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2026</t>
         </is>
       </c>
       <c r="AX19" s="1" t="inlineStr">
@@ -3819,26 +3820,192 @@
       </c>
       <c r="AZ19" s="1" t="inlineStr">
         <is>
-          <t>Дисковые</t>
+          <t>Барабанные</t>
         </is>
       </c>
       <c r="BA19" s="1" t="inlineStr">
         <is>
-          <t>32300</t>
-        </is>
-      </c>
-      <c r="BB19" s="1" t="inlineStr">
-        <is>
-          <t>13600</t>
-        </is>
-      </c>
+          <t>31000</t>
+        </is>
+      </c>
+      <c r="BB19" s="1" t="inlineStr"/>
       <c r="BC19" s="1" t="inlineStr">
         <is>
-          <t>91</t>
+          <t>50</t>
         </is>
       </c>
       <c r="BD19" s="1" t="inlineStr"/>
       <c r="BE19" s="1" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="1" t="inlineStr">
+        <is>
+          <t>Москва, Ижорская ул., 15с2</t>
+        </is>
+      </c>
+      <c r="B20" s="1" t="inlineStr"/>
+      <c r="C20" s="1" t="inlineStr"/>
+      <c r="D20" s="1" t="inlineStr">
+        <is>
+          <t>v-trailer-329d-r0000119</t>
+        </is>
+      </c>
+      <c r="E20" s="1" t="inlineStr"/>
+      <c r="F20" s="1" t="inlineStr"/>
+      <c r="G20" s="1" t="inlineStr"/>
+      <c r="H20" s="1" t="inlineStr"/>
+      <c r="I20" s="1" t="inlineStr"/>
+      <c r="J20" s="1" t="inlineStr"/>
+      <c r="K20" s="1" t="inlineStr"/>
+      <c r="L20" s="1" t="inlineStr">
+        <is>
+          <t>По телефону и в сообщениях</t>
+        </is>
+      </c>
+      <c r="M20" s="1" t="inlineStr">
+        <is>
+          <t>Шторный полуприцеп V-Trailer 329D, 2023 год, в работе, полностью исправен.
+Оси SAF, подъёмная передняя — меньше износ резины и расход на порожняке. Опорное устройство JOST на 24 тонны, шкворень 2 дюйма по ISO 1726. Пол — влагостойкая фанера 30 мм, держит погрузчик до 7,5 тонн. Крыша сдвижная (Sesam/Edscha) — грузить сверху краном или погрузчиком без снятия тента. Двери алюминиевые BPW Smartmaster II, передний и задний портал — стальные, собственной конструкции. Рама облегчённая, с дополнительными усилениями против скручивания. По бортам — корзины под коники, по 7 штук на сторону.
+13,6 × 2,5 × 4 м, 91 м³. Тент плотный: борта 900 г/м², крыша 680 г/м². Полная штора, без бортов — удобно под европаллеты и груз с выступом по высоте.
+Возможна аренда с правом выкупа — уточняйте условия по телефону.</t>
+        </is>
+      </c>
+      <c r="N20" s="1" t="inlineStr">
+        <is>
+          <t>Грузовики и спецтехника</t>
+        </is>
+      </c>
+      <c r="O20" s="1" t="inlineStr">
+        <is>
+          <t>2990000</t>
+        </is>
+      </c>
+      <c r="P20" s="1" t="inlineStr"/>
+      <c r="Q20" s="1" t="inlineStr"/>
+      <c r="R20" s="1" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/v-trailer-329d-r0000119/r2-01.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/v-trailer-329d-r0000119/r2-02.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/v-trailer-329d-r0000119/r2-03.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/v-trailer-329d-r0000119/r2-04.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/v-trailer-329d-r0000119/r2-05.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed-trailers/photos/v-trailer-329d-r0000119/r2-06.jpg</t>
+        </is>
+      </c>
+      <c r="S20" s="1" t="inlineStr"/>
+      <c r="T20" s="1" t="inlineStr"/>
+      <c r="U20" s="1" t="inlineStr">
+        <is>
+          <t>Москва, Ижорская ул., 15с2</t>
+        </is>
+      </c>
+      <c r="V20" s="1" t="inlineStr"/>
+      <c r="W20" s="1" t="inlineStr"/>
+      <c r="X20" s="1" t="inlineStr">
+        <is>
+          <t>Прицепы</t>
+        </is>
+      </c>
+      <c r="Y20" s="1" t="inlineStr">
+        <is>
+          <t>RUB</t>
+        </is>
+      </c>
+      <c r="Z20" s="1" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
+      <c r="AA20" s="1" t="inlineStr"/>
+      <c r="AB20" s="1" t="inlineStr">
+        <is>
+          <t>2990000</t>
+        </is>
+      </c>
+      <c r="AC20" s="1" t="inlineStr">
+        <is>
+          <t>Под заказ</t>
+        </is>
+      </c>
+      <c r="AD20" s="1" t="inlineStr"/>
+      <c r="AE20" s="1" t="inlineStr"/>
+      <c r="AF20" s="1" t="inlineStr"/>
+      <c r="AG20" s="1" t="inlineStr"/>
+      <c r="AH20" s="1" t="inlineStr"/>
+      <c r="AI20" s="1" t="inlineStr"/>
+      <c r="AJ20" s="1" t="inlineStr"/>
+      <c r="AK20" s="1" t="inlineStr"/>
+      <c r="AL20" s="1" t="inlineStr"/>
+      <c r="AM20" s="1" t="inlineStr">
+        <is>
+          <t>С пробегом</t>
+        </is>
+      </c>
+      <c r="AN20" s="1" t="inlineStr"/>
+      <c r="AO20" s="1" t="inlineStr">
+        <is>
+          <t>В наличии</t>
+        </is>
+      </c>
+      <c r="AP20" s="1" t="inlineStr">
+        <is>
+          <t>V-Trailer</t>
+        </is>
+      </c>
+      <c r="AQ20" s="1" t="inlineStr">
+        <is>
+          <t>329</t>
+        </is>
+      </c>
+      <c r="AR20" s="1" t="inlineStr">
+        <is>
+          <t>Полуприцеп</t>
+        </is>
+      </c>
+      <c r="AS20" s="1" t="inlineStr">
+        <is>
+          <t>Шторный</t>
+        </is>
+      </c>
+      <c r="AT20" s="1" t="inlineStr"/>
+      <c r="AU20" s="1" t="inlineStr"/>
+      <c r="AV20" s="1" t="inlineStr">
+        <is>
+          <t>XZFVKRP3DR0000119</t>
+        </is>
+      </c>
+      <c r="AW20" s="1" t="inlineStr">
+        <is>
+          <t>2023</t>
+        </is>
+      </c>
+      <c r="AX20" s="1" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AY20" s="1" t="inlineStr">
+        <is>
+          <t>Пневматическая</t>
+        </is>
+      </c>
+      <c r="AZ20" s="1" t="inlineStr">
+        <is>
+          <t>Дисковые</t>
+        </is>
+      </c>
+      <c r="BA20" s="1" t="inlineStr">
+        <is>
+          <t>32300</t>
+        </is>
+      </c>
+      <c r="BB20" s="1" t="inlineStr">
+        <is>
+          <t>13600</t>
+        </is>
+      </c>
+      <c r="BC20" s="1" t="inlineStr">
+        <is>
+          <t>91</t>
+        </is>
+      </c>
+      <c r="BD20" s="1" t="inlineStr"/>
+      <c r="BE20" s="1" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
B-Trailer: K4-U 2023 (p0002033) 1 690 000 → 1 890 000
</commit_message>
<xml_diff>
--- a/avito-feed-trailers/fleet-trailers.xlsx
+++ b/avito-feed-trailers/fleet-trailers.xlsx
@@ -2811,7 +2811,7 @@
       </c>
       <c r="O12" s="1" t="inlineStr">
         <is>
-          <t>1690000</t>
+          <t>1890000</t>
         </is>
       </c>
       <c r="P12" s="1" t="inlineStr"/>
@@ -2848,7 +2848,7 @@
       <c r="AA12" s="1" t="inlineStr"/>
       <c r="AB12" s="1" t="inlineStr">
         <is>
-          <t>1690000</t>
+          <t>1890000</t>
         </is>
       </c>
       <c r="AC12" s="1" t="inlineStr">

</xml_diff>